<commit_message>
feedback beres, membedakan login
</commit_message>
<xml_diff>
--- a/public/doc/template-peserta-osoca.xlsx
+++ b/public/doc/template-peserta-osoca.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bolou\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/duddy/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6470051A-318F-4A11-B0DA-4BC76797B7FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53BEC9FB-2D16-8E4B-8BF4-FE367F690EAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B39994D4-7263-4FDE-9331-EA3E1EC6B760}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15720" xr2:uid="{B39994D4-7263-4FDE-9331-EA3E1EC6B760}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>No</t>
   </si>
@@ -48,9 +48,6 @@
   </si>
   <si>
     <t>Station</t>
-  </si>
-  <si>
-    <t>Urutan</t>
   </si>
   <si>
     <t>Catur Setiya S</t>
@@ -112,7 +109,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -428,17 +425,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4AC37EF-6132-4013-8A96-FB1B02335EF0}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.5703125" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" customWidth="1"/>
+    <col min="1" max="1" width="4.5" customWidth="1"/>
+    <col min="2" max="2" width="15.5" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -451,16 +447,13 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C2">
         <v>120170099</v>
@@ -468,25 +461,19 @@
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3">
         <v>120170100</v>
       </c>
       <c r="D3">
         <v>1</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>